<commit_message>
docs: standardize public documentation and example workbooks in English
</commit_message>
<xml_diff>
--- a/datasets/synthetic/01_fai/01_fai.xlsx
+++ b/datasets/synthetic/01_fai/01_fai.xlsx
@@ -700,20 +700,20 @@
         <x:v>GaitSPM 1.4</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>FAI sintomático</x:v>
+        <x:v>Symptomatic FAI</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="33" customHeight="1">
       <x:c r="B3" s="14" t="str">
-        <x:v>Datos</x:v>
+        <x:v>Data</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>SINTÉTICOS. 30 casos + 30 controles, 60 participantes únicos.</x:v>
+        <x:v>SYNTHETIC. 30 cases + 30 controls, 60 unique participants.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="33" customHeight="1">
       <x:c r="B4" s="10" t="str">
-        <x:v>Condiciones</x:v>
+        <x:v>Conditions</x:v>
       </x:c>
       <x:c r="C4" s="11" t="n">
         <x:v>1</x:v>
@@ -721,7 +721,7 @@
     </x:row>
     <x:row r="5" ht="33" customHeight="1">
       <x:c r="B5" s="10" t="str">
-        <x:v>Diseño recomendado</x:v>
+        <x:v>Recommended design</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
         <x:v>ttest2</x:v>
@@ -729,66 +729,66 @@
     </x:row>
     <x:row r="6" ht="33" customHeight="1">
       <x:c r="B6" s="10" t="str">
-        <x:v>Grupo para medidas repetidas</x:v>
+        <x:v>Repeated-measures group</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>Control y casos</x:v>
+        <x:v>Control and cases</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="33" customHeight="1">
       <x:c r="B7" s="10" t="str">
-        <x:v>Paso 1</x:v>
+        <x:v>Step 1</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>Inicia GaitSPM y elige CSV / Excel.</x:v>
+        <x:v>Start GaitSPM and select CSV / Excel.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="33" customHeight="1">
       <x:c r="B8" s="10" t="str">
-        <x:v>Paso 2</x:v>
+        <x:v>Step 2</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>Carga este archivo. Se selecciona automáticamente Curves_Wide.</x:v>
+        <x:v>Load this file. Curves_Wide is selected automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="33" customHeight="1">
       <x:c r="B9" s="10" t="str">
-        <x:v>Paso 3</x:v>
+        <x:v>Step 3</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>Revisa ID, grupo, condición, lado y mapeo articular. Aplica el mapeo.</x:v>
+        <x:v>Review ID, group, condition, side and joint mapping. Apply the mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
       <x:c r="B10" s="10" t="str">
-        <x:v>Paso 4</x:v>
+        <x:v>Step 4</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>En modo guiado, revisa el diseño propuesto y ejecuta el análisis.</x:v>
+        <x:v>In guided mode, review the proposed design and run the analysis.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="33" customHeight="1">
       <x:c r="B11" s="10" t="str">
-        <x:v>Paso 5</x:v>
+        <x:v>Step 5</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
-        <x:v>Consulta curvas, clústeres, interpretación, post hoc y exportaciones.</x:v>
+        <x:v>Inspect curves, clusters, interpretation, post hoc comparisons and exports.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="33" customHeight="1">
       <x:c r="B12" s="10" t="str">
-        <x:v>Unidades</x:v>
+        <x:v>Units</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>Grados; nodos 0–100 = porcentaje del ciclo ya segmentado.</x:v>
+        <x:v>Degrees; nodes 0–100 = percentage of the already segmented cycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="33" customHeight="1">
       <x:c r="B13" s="10" t="str">
-        <x:v>Formato</x:v>
+        <x:v>Format</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>Una fila por participante y condición. Los nodos son columnas Variable_0…100.</x:v>
+        <x:v>One row per participant and condition. Nodes are columns Variable_0…100.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="33" customHeight="1">
@@ -796,36 +796,36 @@
         <x:v>Metrics</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>ROM y media del ciclo son fórmulas editables. SPM se calcula en la aplicación.</x:v>
+        <x:v>ROM and cycle mean are editable formulas. SPM is calculated in the application.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
       <x:c r="B15" s="10" t="str">
-        <x:v>Independencia</x:v>
+        <x:v>Independence</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>Las condiciones repetidas NO son nuevos pacientes. IDs conservados.</x:v>
+        <x:v>Repeated conditions are NOT new participants. IDs are preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="33" customHeight="1">
       <x:c r="B16" s="10" t="str">
-        <x:v>Alcance</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>Las formas y covarianzas son simuladas. No representan efectos clínicos demostrados.</x:v>
+        <x:v>Shapes and covariances are simulated. They do not represent demonstrated clinical effects.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="33" customHeight="1">
       <x:c r="B17" s="10" t="str">
-        <x:v>Inferencia</x:v>
+        <x:v>Inference</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
-        <x:v>No significativo no demuestra equivalencia ni ausencia de efecto.</x:v>
+        <x:v>Non-significance does not demonstrate equivalence or absence of an effect.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
       <x:c r="B18" s="10" t="str">
-        <x:v>Semilla</x:v>
+        <x:v>Seed</x:v>
       </x:c>
       <x:c r="C18" s="11" t="n">
         <x:v>260905</x:v>
@@ -833,7 +833,7 @@
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="B19" s="10" t="str">
-        <x:v>Fuente de parámetros</x:v>
+        <x:v>Parameter source</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
         <x:v>Hao et al. (2025), Table 2, FAIS without BDDH</x:v>

</xml_diff>